<commit_message>
Atualização automática 06/04/2026 19:41
</commit_message>
<xml_diff>
--- a/monitor_meta_ads.xlsx
+++ b/monitor_meta_ads.xlsx
@@ -991,8 +991,8 @@
       <c r="K6" s="20" t="n">
         <v>26</v>
       </c>
-      <c r="L6" s="24" t="n">
-        <v>26</v>
+      <c r="L6" s="23" t="n">
+        <v>20</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -1453,7 +1453,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Marcela Cristo</t>
+          <t>Missionario João</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1663,8 +1663,8 @@
       <c r="K21" s="19" t="n">
         <v>43</v>
       </c>
-      <c r="L21" s="25" t="n">
-        <v>53</v>
+      <c r="L21" s="23" t="n">
+        <v>0</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>

</xml_diff>